<commit_message>
Commit from thinkpad on 27/04/2026, 22:49:25
</commit_message>
<xml_diff>
--- a/Entregas PhD/EntregaReview.xlsx
+++ b/Entregas PhD/EntregaReview.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdpds/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdpds/Documents/Obsidian/phd-vault/Entregas PhD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6252CA69-CFF6-BC44-B206-C37C8851C655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6ADEF3-1388-324D-8B74-68E69CEDC45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{D4FC6CEF-DE37-9F4F-9AF8-564C0215D0C0}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29840" windowHeight="16960" xr2:uid="{D4FC6CEF-DE37-9F4F-9AF8-564C0215D0C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
   <si>
     <t>Ranking</t>
   </si>
@@ -68,9 +68,6 @@
     <t>CiteScore</t>
   </si>
   <si>
-    <t>Submission to first Decision</t>
-  </si>
-  <si>
     <t>Submission to decision after review</t>
   </si>
   <si>
@@ -101,33 +98,6 @@
     <t>Q1</t>
   </si>
   <si>
-    <t>Renewable and Sustainable Energy Reviews</t>
-  </si>
-  <si>
-    <t>Elsevier</t>
-  </si>
-  <si>
-    <t>https://www.sciencedirect.com/journal/renewable-and-sustainable-energy-reviews</t>
-  </si>
-  <si>
-    <t>2 days</t>
-  </si>
-  <si>
-    <t>97 days</t>
-  </si>
-  <si>
-    <t>172 days</t>
-  </si>
-  <si>
-    <t>9 days</t>
-  </si>
-  <si>
-    <t>38.0</t>
-  </si>
-  <si>
-    <t>16.3</t>
-  </si>
-  <si>
     <t>WIREs Data Mining and Knowledge Discovery</t>
   </si>
   <si>
@@ -155,84 +125,60 @@
     <t>Hybrid</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">prioritizes the </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>methodological</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> shift you propose: how to structure raw behavioral signals into evolved, reasoned human-centric models</t>
-    </r>
-  </si>
-  <si>
-    <t>Knowledge discovery in complex environments; high-level data modeling; AI architectures for reasoning over user intent.</t>
-  </si>
-  <si>
-    <t>State-of-the-art surveys on data mining; human-centric AI; evolving user preference frameworks.</t>
-  </si>
-  <si>
-    <t>Sustainable built environments; human-dimension in energy systems; smart building policy and occupant behavior.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">If the review emphasizes the </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>impact</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> of modeling "personas" on energy efficiency and sustainable interaction, this is the highest-impact venue.</t>
-    </r>
-  </si>
-  <si>
-    <t>Ideal due to the nature of the review, which feeds on several areas of interest</t>
+    <t>Artificial Intelligence Review</t>
+  </si>
+  <si>
+    <t>Open Access</t>
+  </si>
+  <si>
+    <t>Springer</t>
+  </si>
+  <si>
+    <t>https://link.springer.com/journal/10462</t>
+  </si>
+  <si>
+    <t>13.9</t>
+  </si>
+  <si>
+    <t>12 days</t>
+  </si>
+  <si>
+    <t>26.3</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>15.7</t>
+  </si>
+  <si>
+    <t>Submission to first decision</t>
+  </si>
+  <si>
+    <t>Abrange reviews de métodos de IA com scope interdisciplinar, nomeadamente representação de conhecimento, user modeling e sistemas inteligentes.</t>
+  </si>
+  <si>
+    <t>Alinhado com a mudança metodológica que este review supõe: como estruturar sinais comportamentais brutos em modelos evoluídos, racionais e centrados no ser humano.</t>
+  </si>
+  <si>
+    <t>Ideal devido tema da revisão, que abrange diversas áreas de interesse, especialmente na captação de dados do utilizador e como os representar.</t>
+  </si>
+  <si>
+    <t>State of the art reviews em IA</t>
+  </si>
+  <si>
+    <t>Descoberta de conhecimento em ambientes complexos; modelação de dados; arquiteturas de IA para raciocínio sobre a intenção do utilizador.</t>
+  </si>
+  <si>
+    <t>State of the art em data mining; IA centrada no ser humano; evolução dos modelos de preferências do utilizador.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -605,9 +551,9 @@
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="23.5" customWidth="1"/>
-    <col min="6" max="6" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.1640625" customWidth="1"/>
     <col min="7" max="7" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -648,127 +594,151 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
-        <v>14</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:15" ht="59" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="136" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F2" t="s">
-        <v>39</v>
+      <c r="F2" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>35</v>
       </c>
       <c r="O2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="51" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="136" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" t="s">
-        <v>40</v>
+        <v>39</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="I3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>35</v>
       </c>
       <c r="L3" t="s">
         <v>35</v>
       </c>
       <c r="M3" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
       </c>
       <c r="O3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="102" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" ht="119" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
-      </c>
       <c r="I4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="J4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K4" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="L4" t="s">
         <v>25</v>
@@ -776,8 +746,11 @@
       <c r="M4" t="s">
         <v>26</v>
       </c>
+      <c r="N4" t="s">
+        <v>35</v>
+      </c>
       <c r="O4" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit from thinkpad on 27/04/2026, 23:11:17
</commit_message>
<xml_diff>
--- a/Entregas PhD/EntregaReview.xlsx
+++ b/Entregas PhD/EntregaReview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdpds/Documents/Obsidian/phd-vault/Entregas PhD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD64F626-8D89-9A4D-A2B1-A2D3036B2C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530BC7F3-A46B-2143-B0B5-A9540DED26F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29840" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -304,7 +304,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -312,24 +312,156 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.34998626667073579"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -340,6 +472,30 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08F0A559-0754-0249-A5E5-BC99D634C690}" name="Tabela1" displayName="Tabela1" ref="A1:O8" totalsRowShown="0">
+  <autoFilter ref="A1:O8" xr:uid="{08F0A559-0754-0249-A5E5-BC99D634C690}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{C63AF7E6-E620-F04A-A1DB-3E2D9772B8A2}" name="Ranking"/>
+    <tableColumn id="2" xr3:uid="{A3045780-643D-0446-81F6-85840C9AD8D4}" name="Journal"/>
+    <tableColumn id="3" xr3:uid="{834542A2-8D85-8D48-BEA0-490C85614A26}" name="Publisher"/>
+    <tableColumn id="4" xr3:uid="{216BDDE6-3EA3-684E-8A4C-D14EF83B1BEF}" name="Webpage"/>
+    <tableColumn id="5" xr3:uid="{75F799C0-E817-FD43-AA24-176BCED5F940}" name="Why this journal" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{4C964E92-14DB-714B-B5EA-0323B695AB0D}" name="Scope" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{B2687B74-97FE-A649-95E1-FF1A7DA68E0B}" name="Quartil"/>
+    <tableColumn id="8" xr3:uid="{3D657B1F-9108-AF4A-B9BF-A06F01030D64}" name="IF"/>
+    <tableColumn id="9" xr3:uid="{015A05CE-1767-C047-9D7E-78C135AC018F}" name="CiteScore"/>
+    <tableColumn id="10" xr3:uid="{CAF09DF6-4EEA-A34E-8639-1AE9DB7D6A28}" name="Submission to first decision"/>
+    <tableColumn id="11" xr3:uid="{22521360-4B5D-BF44-8A81-8A504A4510C0}" name="Submission to decision after review"/>
+    <tableColumn id="12" xr3:uid="{378E52F1-CD46-4944-8E63-EE117397E736}" name="Submission to acceptance"/>
+    <tableColumn id="13" xr3:uid="{61DEE2C5-41E5-C941-B560-2A00AECF26B8}" name="Acceptance to online publication"/>
+    <tableColumn id="14" xr3:uid="{38D58924-B902-3A49-BB6E-41A29B8E9575}" name="Submission to publication"/>
+    <tableColumn id="15" xr3:uid="{4AE19BBE-191C-9B4B-AB65-716EDC2EF05F}" name="Type (open access /hybrid)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium18" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -662,21 +818,21 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1640625" customWidth="1"/>
     <col min="2" max="2" width="45" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.1640625" customWidth="1"/>
     <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.1640625" customWidth="1"/>
+    <col min="8" max="8" width="5" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" customWidth="1"/>
+    <col min="10" max="10" width="26.33203125" customWidth="1"/>
+    <col min="11" max="11" width="32.5" customWidth="1"/>
+    <col min="12" max="12" width="25.1640625" customWidth="1"/>
+    <col min="13" max="13" width="30.1640625" customWidth="1"/>
+    <col min="14" max="14" width="24.6640625" customWidth="1"/>
+    <col min="15" max="15" width="25.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -730,140 +886,140 @@
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O2" s="2" t="s">
+      <c r="K2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="136" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+      <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" s="2" t="s">
+      <c r="J3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="O3" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="119" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4" s="10">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="2" t="s">
+      <c r="K4" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="13" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1057,5 +1213,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Commit from thinkpad on 27/04/2026, 23:26:18
</commit_message>
<xml_diff>
--- a/Entregas PhD/EntregaReview.xlsx
+++ b/Entregas PhD/EntregaReview.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rdpds/Documents/Obsidian/phd-vault/Entregas PhD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E074A805-572B-074B-81C0-3A06150AC10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35593809-CF48-FE4D-8414-F3CD393010E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29840" windowHeight="16960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29840" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Folha1" sheetId="1" r:id="rId1"/>
-    <sheet name="Folha2" sheetId="2" r:id="rId2"/>
+    <sheet name="Folha2" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="95">
   <si>
     <t>Ranking</t>
   </si>
@@ -278,51 +277,6 @@
     <t>230 days</t>
   </si>
   <si>
-    <t>Coluna1</t>
-  </si>
-  <si>
-    <t>Coluna2</t>
-  </si>
-  <si>
-    <t>Coluna3</t>
-  </si>
-  <si>
-    <t>Coluna4</t>
-  </si>
-  <si>
-    <t>Coluna5</t>
-  </si>
-  <si>
-    <t>Coluna6</t>
-  </si>
-  <si>
-    <t>Coluna7</t>
-  </si>
-  <si>
-    <t>Coluna8</t>
-  </si>
-  <si>
-    <t>Coluna9</t>
-  </si>
-  <si>
-    <t>Coluna10</t>
-  </si>
-  <si>
-    <t>Coluna11</t>
-  </si>
-  <si>
-    <t>Coluna12</t>
-  </si>
-  <si>
-    <t>Coluna13</t>
-  </si>
-  <si>
-    <t>Coluna14</t>
-  </si>
-  <si>
-    <t>Coluna15</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome: </t>
   </si>
   <si>
@@ -348,6 +302,9 @@
   </si>
   <si>
     <t>Human-centric intelligent environments: From signals to adaptive environments</t>
+  </si>
+  <si>
+    <t>Data: 27/04/2026</t>
   </si>
 </sst>
 </file>
@@ -415,11 +372,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -433,14 +387,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -451,30 +398,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{08F0A559-0754-0249-A5E5-BC99D634C690}" name="Tabela1" displayName="Tabela1" ref="A1:O11" totalsRowShown="0">
-  <autoFilter ref="A1:O11" xr:uid="{08F0A559-0754-0249-A5E5-BC99D634C690}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{C63AF7E6-E620-F04A-A1DB-3E2D9772B8A2}" name="Coluna1"/>
-    <tableColumn id="2" xr3:uid="{A3045780-643D-0446-81F6-85840C9AD8D4}" name="Coluna2"/>
-    <tableColumn id="3" xr3:uid="{834542A2-8D85-8D48-BEA0-490C85614A26}" name="Coluna3"/>
-    <tableColumn id="4" xr3:uid="{216BDDE6-3EA3-684E-8A4C-D14EF83B1BEF}" name="Coluna4"/>
-    <tableColumn id="5" xr3:uid="{75F799C0-E817-FD43-AA24-176BCED5F940}" name="Coluna5" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{4C964E92-14DB-714B-B5EA-0323B695AB0D}" name="Coluna6" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{B2687B74-97FE-A649-95E1-FF1A7DA68E0B}" name="Coluna7"/>
-    <tableColumn id="8" xr3:uid="{3D657B1F-9108-AF4A-B9BF-A06F01030D64}" name="Coluna8"/>
-    <tableColumn id="9" xr3:uid="{015A05CE-1767-C047-9D7E-78C135AC018F}" name="Coluna9"/>
-    <tableColumn id="10" xr3:uid="{CAF09DF6-4EEA-A34E-8639-1AE9DB7D6A28}" name="Coluna10"/>
-    <tableColumn id="11" xr3:uid="{22521360-4B5D-BF44-8A81-8A504A4510C0}" name="Coluna11"/>
-    <tableColumn id="12" xr3:uid="{378E52F1-CD46-4944-8E63-EE117397E736}" name="Coluna12"/>
-    <tableColumn id="13" xr3:uid="{61DEE2C5-41E5-C941-B560-2A00AECF26B8}" name="Coluna13"/>
-    <tableColumn id="14" xr3:uid="{38D58924-B902-3A49-BB6E-41A29B8E9575}" name="Coluna14"/>
-    <tableColumn id="15" xr3:uid="{4AE19BBE-191C-9B4B-AB65-716EDC2EF05F}" name="Coluna15"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium18" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -793,91 +716,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.1640625" customWidth="1"/>
-    <col min="2" max="2" width="45" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
-    <col min="4" max="4" width="11.1640625" customWidth="1"/>
-    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1640625" customWidth="1"/>
-    <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" customWidth="1"/>
-    <col min="11" max="11" width="32.5" customWidth="1"/>
-    <col min="12" max="12" width="25.1640625" customWidth="1"/>
-    <col min="13" max="13" width="30.1640625" customWidth="1"/>
-    <col min="14" max="14" width="24.6640625" customWidth="1"/>
-    <col min="15" max="15" width="25.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-      <c r="F1" t="s">
-        <v>90</v>
-      </c>
-      <c r="G1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H1" t="s">
-        <v>92</v>
-      </c>
-      <c r="I1" t="s">
-        <v>93</v>
-      </c>
-      <c r="J1" t="s">
-        <v>94</v>
-      </c>
-      <c r="K1" t="s">
-        <v>95</v>
-      </c>
-      <c r="L1" t="s">
-        <v>96</v>
-      </c>
-      <c r="M1" t="s">
-        <v>97</v>
-      </c>
-      <c r="N1" t="s">
-        <v>98</v>
-      </c>
-      <c r="O1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="136" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:15" ht="136" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:15" ht="119" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B8E522-547A-BA4D-AC32-863A5D9B4D77}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -899,425 +741,429 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>100</v>
+      <c r="A1" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="6">
+        <v>86</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="5">
         <v>1190979</v>
+      </c>
+      <c r="F1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>103</v>
+      <c r="A2" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
+        <v>93</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>104</v>
+      <c r="A3" s="4" t="s">
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6"/>
+        <v>92</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>105</v>
+      <c r="A4" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>1</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O7" s="2" t="s">
+      <c r="K7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="51" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O8" s="2" t="s">
+      <c r="J8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>3</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O9" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="102" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>4</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="102" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>5</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O11" s="2" t="s">
+      <c r="J11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O11" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="68" x14ac:dyDescent="0.2">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>6</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L12" s="2" t="s">
+      <c r="K12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="M12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="N12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="O12" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="85" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>7</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="K13" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="M13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="N13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="O13" s="1" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="64" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>